<commit_message>
Redesign invoice: move issuer to header top-right, refresh styling
- 発行者情報をヘッダー右上のカードに移動
- ヘッダー背景にドットパターン・グロー装飾を追加
- Excel版も同様にヘッダーレイアウトを再設計

https://claude.ai/code/session_01EYbGt2cY4jePpiqNLd4Beb
</commit_message>
<xml_diff>
--- a/請求書_INV-20260525-001.xlsx
+++ b/請求書_INV-20260525-001.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="¥#,##0"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,53 +32,8 @@
     <font>
       <name val="游ゴシック"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="20"/>
-    </font>
-    <font>
-      <name val="游ゴシック"/>
-      <i val="1"/>
-      <color rgb="00AAAACC"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="游ゴシック"/>
-      <b val="1"/>
-      <color rgb="00888888"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="游ゴシック"/>
-      <b val="1"/>
-      <color rgb="00764BA2"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="游ゴシック"/>
-      <color rgb="001A1A2E"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="游ゴシック"/>
-      <b val="1"/>
-      <color rgb="00764BA2"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="游ゴシック"/>
-      <b val="1"/>
-      <color rgb="001A1A2E"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="游ゴシック"/>
-      <color rgb="001A1A2E"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="游ゴシック"/>
-      <color rgb="00AAAACC"/>
-      <sz val="10"/>
+      <color rgb="00A5B4FC"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="游ゴシック"/>
@@ -88,8 +43,48 @@
     </font>
     <font>
       <name val="游ゴシック"/>
-      <color rgb="00888888"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <b val="1"/>
+      <color rgb="00A5B4FC"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <color rgb="00CCCCCC"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <color rgb="00A5B4FC"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <b val="1"/>
+      <color rgb="00764BA2"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <b val="1"/>
+      <color rgb="001A1A2E"/>
+      <sz val="17"/>
     </font>
     <font>
       <name val="游ゴシック"/>
@@ -98,33 +93,61 @@
     </font>
     <font>
       <name val="游ゴシック"/>
-      <color rgb="00764BA2"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="游ゴシック"/>
-      <b val="1"/>
-      <color rgb="001A1A3E"/>
-      <sz val="12"/>
+      <color rgb="008899CC"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="游ゴシック"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="游ゴシック"/>
-      <color rgb="001A1A3E"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <b val="1"/>
+      <color rgb="00764BA2"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <color rgb="00999999"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <color rgb="001A1A2E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <color rgb="00764BA2"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="游ゴシック"/>
-      <color rgb="00888888"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="00999999"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <color rgb="001A1245"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="游ゴシック"/>
+      <i val="1"/>
+      <color rgb="00CCCCCC"/>
+      <sz val="8"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -133,7 +156,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A1A3E"/>
+        <fgColor rgb="000A0818"/>
       </patternFill>
     </fill>
     <fill>
@@ -143,7 +166,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F3F0FB"/>
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A1245"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F2FC"/>
       </patternFill>
     </fill>
     <fill>
@@ -153,11 +186,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00FAF8FF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -167,104 +200,131 @@
     </border>
     <border>
       <bottom style="medium">
-        <color rgb="00764BA2"/>
+        <color rgb="001A1245"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D0C8F0"/>
+        <color rgb="00E2D9F3"/>
       </left>
       <right style="thin">
-        <color rgb="00D0C8F0"/>
+        <color rgb="00E2D9F3"/>
       </right>
       <top style="thin">
-        <color rgb="00D0C8F0"/>
+        <color rgb="00E2D9F3"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D0C8F0"/>
+        <color rgb="00E2D9F3"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="001A1245"/>
+      </left>
+      <right style="thin">
+        <color rgb="001A1245"/>
+      </right>
+      <top style="thin">
+        <color rgb="001A1245"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="001A1245"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -632,294 +692,362 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="3" customWidth="1" min="8" max="8"/>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="2" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="8" customHeight="1"/>
-    <row r="2" ht="36" customHeight="1">
+    <row r="1" ht="6" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>INVOICE</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>ISSUED BY</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="n"/>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
           <t>請 求 書</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Invoice</t>
-        </is>
-      </c>
-      <c r="H2" s="1" t="n"/>
-    </row>
-    <row r="3" ht="5" customHeight="1">
-      <c r="A3" s="4" t="n"/>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="4" t="n"/>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>請求書番号</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>可知 優也</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="1" t="n"/>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>愛知県名古屋市昭和区壇溪通1丁目7番地</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="1" t="n"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>INV-20260525-001</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>発行日</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="1" t="n"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>アンシェリーナ106</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>2026年5月25日</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="10" customHeight="1"/>
-    <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>■ 請求先</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="9" t="inlineStr">
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>TEL: 080-6925-9411</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="n"/>
+    </row>
+    <row r="7" ht="4" customHeight="1">
+      <c r="A7" s="9" t="n"/>
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>免税事業者 · 登録番号なし</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
+    </row>
+    <row r="8" ht="6" customHeight="1"/>
+    <row r="9" ht="16" customHeight="1">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>BILL TO  /  請求先</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>合同会社 Frigus　御中</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="10" t="inlineStr"/>
-    </row>
-    <row r="10" ht="10" customHeight="1"/>
-    <row r="11" ht="38" customHeight="1">
-      <c r="B11" s="11" t="inlineStr">
+    <row r="11" ht="14" customHeight="1">
+      <c r="B11" s="13" t="inlineStr"/>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="14" t="n"/>
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>ご請求金額（税込）</t>
         </is>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E12" s="16" t="n">
         <v>202306</v>
       </c>
-    </row>
-    <row r="12" ht="10" customHeight="1"/>
-    <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="13" t="inlineStr">
+      <c r="H12" s="14" t="n"/>
+    </row>
+    <row r="13" ht="6" customHeight="1"/>
+    <row r="14" ht="30" customHeight="1">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>日付</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>数量</t>
         </is>
       </c>
-      <c r="F13" s="13" t="inlineStr">
+      <c r="E14" s="17" t="inlineStr">
         <is>
           <t>単位</t>
         </is>
       </c>
-      <c r="G13" s="15" t="inlineStr">
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>税区分</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
         <is>
           <t>金額</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="B14" s="16" t="inlineStr">
+    <row r="15" ht="6" customHeight="1"/>
+    <row r="16" ht="26" customHeight="1">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>2026年5月25日</t>
         </is>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>Goo Property Singapore Pte. Ltd.社からの保全費（2026年2月預かり金より）</t>
         </is>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="D16" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="E16" s="22" t="inlineStr">
         <is>
           <t>式</t>
         </is>
       </c>
-      <c r="G14" s="19" t="inlineStr">
+      <c r="F16" s="23" t="inlineStr">
         <is>
           <t>対象外</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="14" customHeight="1"/>
-    <row r="16" ht="22" customHeight="1">
-      <c r="E16" s="20" t="inlineStr">
+      <c r="G16" s="24" t="n">
+        <v>202306</v>
+      </c>
+    </row>
+    <row r="17" ht="6" customHeight="1"/>
+    <row r="18" ht="20" customHeight="1">
+      <c r="E18" s="25" t="inlineStr">
         <is>
           <t>小計</t>
         </is>
       </c>
-      <c r="G16" s="21" t="n">
+      <c r="G18" s="26" t="inlineStr">
+        <is>
+          <t>¥202,306</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="E19" s="25" t="inlineStr">
+        <is>
+          <t>消費税</t>
+        </is>
+      </c>
+      <c r="G19" s="26" t="inlineStr">
+        <is>
+          <t>¥0（対象外）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>合　計</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
         <v>202306</v>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="E17" s="20" t="inlineStr">
-        <is>
-          <t>消費税</t>
-        </is>
-      </c>
-      <c r="G17" s="22" t="inlineStr">
-        <is>
-          <t>¥0（対象外）</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="E18" s="23" t="inlineStr">
-        <is>
-          <t>合計</t>
-        </is>
-      </c>
-      <c r="G18" s="24" t="n">
-        <v>202306</v>
-      </c>
-    </row>
-    <row r="19" ht="14" customHeight="1"/>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>■ お振込先</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="25" t="inlineStr">
+    <row r="21" ht="6" customHeight="1"/>
+    <row r="22" ht="16" customHeight="1">
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>BANK TRANSFER  /  お振込先</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="30" t="inlineStr">
         <is>
           <t>銀行名</t>
         </is>
       </c>
-      <c r="C21" s="26" t="inlineStr">
+      <c r="C23" s="31" t="inlineStr">
         <is>
           <t>楽天銀行</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="14" customHeight="1">
-      <c r="B22" s="25" t="inlineStr">
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="30" t="inlineStr">
         <is>
           <t>支店名</t>
         </is>
       </c>
-      <c r="C22" s="26" t="inlineStr">
+      <c r="C24" s="31" t="inlineStr">
         <is>
           <t>ボレロ支店</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="25" t="inlineStr">
+    <row r="25" ht="20" customHeight="1">
+      <c r="B25" s="30" t="inlineStr">
         <is>
           <t>口座種別</t>
         </is>
       </c>
-      <c r="C23" s="26" t="inlineStr">
+      <c r="C25" s="31" t="inlineStr">
         <is>
           <t>普通預金</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="14" customHeight="1">
-      <c r="B24" s="25" t="inlineStr">
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="30" t="inlineStr">
         <is>
           <t>口座番号</t>
         </is>
       </c>
-      <c r="C24" s="26" t="inlineStr">
+      <c r="C26" s="31" t="inlineStr">
         <is>
           <t>4541728</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="25" t="inlineStr">
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="30" t="inlineStr">
         <is>
           <t>口座名義</t>
         </is>
       </c>
-      <c r="C25" s="26" t="inlineStr">
+      <c r="C27" s="31" t="inlineStr">
         <is>
           <t>カチユウヤ</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="14" customHeight="1"/>
-    <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>■ 発行者</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="14" customHeight="1">
-      <c r="B28" s="27" t="inlineStr">
-        <is>
-          <t>可知 優也　|　愛知県名古屋市昭和区壇溪通1丁目7番地 アンシェリーナ106　|　TEL: 080-6925-9411　|　免税事業者</t>
-        </is>
-      </c>
-    </row>
+    <row r="28" ht="6" customHeight="1"/>
+    <row r="29" ht="16" customHeight="1">
+      <c r="B29" s="32" t="inlineStr">
+        <is>
+          <t>ご不明な点はお気軽にご連絡ください。  TEL: 080-6925-9411</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="6" customHeight="1"/>
   </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B9:E9"/>
+  <mergeCells count="28">
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="C6:D6"/>
     <mergeCell ref="C24:G24"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="B28:G28"/>
-    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="B6"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="B5"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="E19:F19"/>
     <mergeCell ref="C25:G25"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="B20:G20"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="C14"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="E12:G12"/>
     <mergeCell ref="C23:G23"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B27:G27"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B10:E10"/>
     <mergeCell ref="E18:F18"/>
     <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B11:G11"/>
   </mergeCells>
-  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Move issuer panel to right edge with diagonal cut design
- 発行者情報をヘッダー右端の斜めカットパネルに配置
- No./Dateはタイトル直下の左側に固定
- Excel版も同様にF-H列右端に発行者ブロックを配置

https://claude.ai/code/session_01EYbGt2cY4jePpiqNLd4Beb
</commit_message>
<xml_diff>
--- a/請求書_INV-20260525-001.xlsx
+++ b/請求書_INV-20260525-001.xlsx
@@ -10,7 +10,7 @@
     <sheet name="請求書" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'請求書'!$A$1:$H$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'請求書'!$A$1:$I$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -39,7 +39,7 @@
       <name val="游ゴシック"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="22"/>
+      <sz val="20"/>
     </font>
     <font>
       <name val="游ゴシック"/>
@@ -62,7 +62,7 @@
       <name val="游ゴシック"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="游ゴシック"/>
@@ -71,7 +71,7 @@
     </font>
     <font>
       <name val="游ゴシック"/>
-      <color rgb="00A5B4FC"/>
+      <color rgb="00555577"/>
       <sz val="7"/>
     </font>
     <font>
@@ -84,7 +84,7 @@
       <name val="游ゴシック"/>
       <b val="1"/>
       <color rgb="001A1A2E"/>
-      <sz val="17"/>
+      <sz val="16"/>
     </font>
     <font>
       <name val="游ゴシック"/>
@@ -100,7 +100,7 @@
       <name val="游ゴシック"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="20"/>
+      <sz val="18"/>
     </font>
     <font>
       <name val="游ゴシック"/>
@@ -147,7 +147,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -162,6 +162,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00764BA2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F0C30"/>
       </patternFill>
     </fill>
     <fill>
@@ -238,54 +243,55 @@
   <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -297,31 +303,28 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="18" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -692,17 +695,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="2" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="2" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="6" customHeight="1">
@@ -711,165 +715,165 @@
       <c r="C1" s="1" t="n"/>
       <c r="D1" s="1" t="n"/>
       <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-    </row>
-    <row r="2" ht="18" customHeight="1">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="1" t="n"/>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>INVOICE</t>
         </is>
       </c>
       <c r="E2" s="1" t="n"/>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>ISSUED BY</t>
         </is>
       </c>
-      <c r="H2" s="1" t="n"/>
-    </row>
-    <row r="3" ht="32" customHeight="1">
+      <c r="I2" s="1" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="1" t="n"/>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>請 求 書</t>
         </is>
       </c>
       <c r="E3" s="1" t="n"/>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>可知 優也</t>
         </is>
       </c>
-      <c r="H3" s="1" t="n"/>
-    </row>
-    <row r="4" ht="20" customHeight="1">
+      <c r="I3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
       <c r="A4" s="1" t="n"/>
-      <c r="B4" s="1" t="n"/>
-      <c r="C4" s="1" t="n"/>
-      <c r="D4" s="1" t="n"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>INV-20260525-001</t>
+        </is>
+      </c>
       <c r="E4" s="1" t="n"/>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>愛知県名古屋市昭和区壇溪通1丁目7番地</t>
         </is>
       </c>
-      <c r="H4" s="1" t="n"/>
+      <c r="I4" s="1" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="1" t="n"/>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>INV-20260525-001</t>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>2026年5月25日</t>
         </is>
       </c>
       <c r="E5" s="1" t="n"/>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>アンシェリーナ106</t>
         </is>
       </c>
-      <c r="H5" s="1" t="n"/>
+      <c r="I5" s="1" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="1" t="n"/>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>DATE</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>2026年5月25日</t>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>免税事業者 · 登録番号なし</t>
         </is>
       </c>
       <c r="E6" s="1" t="n"/>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>TEL: 080-6925-9411</t>
         </is>
       </c>
-      <c r="H6" s="1" t="n"/>
+      <c r="I6" s="1" t="n"/>
     </row>
     <row r="7" ht="4" customHeight="1">
-      <c r="A7" s="9" t="n"/>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>免税事業者 · 登録番号なし</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="9" t="n"/>
-    </row>
-    <row r="8" ht="6" customHeight="1"/>
-    <row r="9" ht="16" customHeight="1">
-      <c r="B9" s="11" t="inlineStr">
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="11" t="n"/>
+      <c r="I7" s="11" t="n"/>
+    </row>
+    <row r="8" ht="8" customHeight="1">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>BILL TO  /  請求先</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="12" t="inlineStr">
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>合同会社 Frigus　御中</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="14" customHeight="1">
-      <c r="B11" s="13" t="inlineStr"/>
-    </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="14" t="n"/>
-      <c r="B12" s="15" t="inlineStr">
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="14" t="inlineStr"/>
+    </row>
+    <row r="11" ht="10" customHeight="1"/>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="15" t="n"/>
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>ご請求金額（税込）</t>
         </is>
       </c>
-      <c r="E12" s="16" t="n">
+      <c r="F12" s="17" t="n">
         <v>202306</v>
       </c>
-      <c r="H12" s="14" t="n"/>
+      <c r="I12" s="15" t="n"/>
     </row>
     <row r="13" ht="6" customHeight="1"/>
-    <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="17" t="inlineStr">
+    <row r="14" ht="26" customHeight="1">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>日付</t>
         </is>
       </c>
-      <c r="C14" s="18" t="inlineStr">
+      <c r="C14" s="19" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="E14" s="18" t="inlineStr">
         <is>
           <t>数量</t>
         </is>
       </c>
-      <c r="E14" s="17" t="inlineStr">
+      <c r="F14" s="18" t="inlineStr">
         <is>
           <t>単位</t>
         </is>
       </c>
-      <c r="F14" s="17" t="inlineStr">
+      <c r="G14" s="18" t="inlineStr">
         <is>
           <t>税区分</t>
         </is>
       </c>
-      <c r="G14" s="19" t="inlineStr">
+      <c r="H14" s="20" t="inlineStr">
         <is>
           <t>金額</t>
         </is>
@@ -877,77 +881,77 @@
     </row>
     <row r="15" ht="6" customHeight="1"/>
     <row r="16" ht="26" customHeight="1">
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>2026年5月25日</t>
         </is>
       </c>
-      <c r="C16" s="21" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>Goo Property Singapore Pte. Ltd.社からの保全費（2026年2月預かり金より）</t>
         </is>
       </c>
-      <c r="D16" s="22" t="n">
+      <c r="E16" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="22" t="inlineStr">
+      <c r="F16" s="23" t="inlineStr">
         <is>
           <t>式</t>
         </is>
       </c>
-      <c r="F16" s="23" t="inlineStr">
+      <c r="G16" s="24" t="inlineStr">
         <is>
           <t>対象外</t>
         </is>
       </c>
-      <c r="G16" s="24" t="n">
+      <c r="H16" s="25" t="n">
         <v>202306</v>
       </c>
     </row>
     <row r="17" ht="6" customHeight="1"/>
-    <row r="18" ht="20" customHeight="1">
-      <c r="E18" s="25" t="inlineStr">
+    <row r="18" ht="18" customHeight="1">
+      <c r="F18" s="26" t="inlineStr">
         <is>
           <t>小計</t>
         </is>
       </c>
-      <c r="G18" s="26" t="inlineStr">
+      <c r="H18" s="27" t="inlineStr">
         <is>
           <t>¥202,306</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="E19" s="25" t="inlineStr">
+    <row r="19" ht="18" customHeight="1">
+      <c r="F19" s="26" t="inlineStr">
         <is>
           <t>消費税</t>
         </is>
       </c>
-      <c r="G19" s="26" t="inlineStr">
+      <c r="H19" s="27" t="inlineStr">
         <is>
           <t>¥0（対象外）</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="E20" s="27" t="inlineStr">
+    <row r="20" ht="18" customHeight="1">
+      <c r="F20" s="28" t="inlineStr">
         <is>
           <t>合　計</t>
         </is>
       </c>
-      <c r="G20" s="28" t="n">
+      <c r="H20" s="29" t="n">
         <v>202306</v>
       </c>
     </row>
     <row r="21" ht="6" customHeight="1"/>
     <row r="22" ht="16" customHeight="1">
-      <c r="B22" s="29" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>BANK TRANSFER  /  お振込先</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="20" customHeight="1">
+    <row r="23" ht="18" customHeight="1">
       <c r="B23" s="30" t="inlineStr">
         <is>
           <t>銀行名</t>
@@ -959,7 +963,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
+    <row r="24" ht="18" customHeight="1">
       <c r="B24" s="30" t="inlineStr">
         <is>
           <t>支店名</t>
@@ -971,7 +975,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1">
+    <row r="25" ht="18" customHeight="1">
       <c r="B25" s="30" t="inlineStr">
         <is>
           <t>口座種別</t>
@@ -983,7 +987,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="20" customHeight="1">
+    <row r="26" ht="18" customHeight="1">
       <c r="B26" s="30" t="inlineStr">
         <is>
           <t>口座番号</t>
@@ -995,7 +999,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
+    <row r="27" ht="18" customHeight="1">
       <c r="B27" s="30" t="inlineStr">
         <is>
           <t>口座名義</t>
@@ -1008,44 +1012,42 @@
       </c>
     </row>
     <row r="28" ht="6" customHeight="1"/>
-    <row r="29" ht="16" customHeight="1">
+    <row r="29" ht="14" customHeight="1">
       <c r="B29" s="32" t="inlineStr">
         <is>
           <t>ご不明な点はお気軽にご連絡ください。  TEL: 080-6925-9411</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="6" customHeight="1"/>
   </sheetData>
-  <mergeCells count="28">
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C24:G24"/>
+  <mergeCells count="27">
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="F19:G19"/>
     <mergeCell ref="C5:D5"/>
-    <mergeCell ref="B6"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="B5"/>
-    <mergeCell ref="B29:G29"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="B9:G9"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="C14"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="E12:G12"/>
-    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C27:H27"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="B8:H8"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="B29:H29"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="F12:H12"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B11:G11"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>